<commit_message>
Fix: Alteração no riqu
</commit_message>
<xml_diff>
--- a/Arquivos-Escopo/Requisitos_Fazenda (1).xlsx
+++ b/Arquivos-Escopo/Requisitos_Fazenda (1).xlsx
@@ -1,16 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
-  <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20384"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DTG-2025\Desktop\AgroFlux2026\Arquivos-Escopo\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65264BA7-9048-4346-A331-E118A46B2C7A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="16380" windowHeight="8196" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Planilha1" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
+  <calcPr calcId="0" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="CalcA1ExcelA1"/>
@@ -22,192 +27,170 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="40">
   <si>
-    <t xml:space="preserve">REQUISITOS FUNCIONAIS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DESCRIÇÃO DO REQUISITO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CLASSIFICAÇÃO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RF 01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">O SISTEMA DEVERÁ CONTER PÁGINAS DE LOGIN PARA FUNCIONÁRIOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ESSENCIAL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RF 02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">O SISTEMA DEVERÁ CONTER UMA
+    <t>REQUISITOS FUNCIONAIS</t>
+  </si>
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>DESCRIÇÃO DO REQUISITO</t>
+  </si>
+  <si>
+    <t>CLASSIFICAÇÃO</t>
+  </si>
+  <si>
+    <t>RF 01</t>
+  </si>
+  <si>
+    <t>O SISTEMA DEVERÁ CONTER PÁGINAS DE LOGIN PARA FUNCIONÁRIOS</t>
+  </si>
+  <si>
+    <t>ESSENCIAL</t>
+  </si>
+  <si>
+    <t>RF 02</t>
+  </si>
+  <si>
+    <t>O SISTEMA DEVERÁ CONTER UMA
 PÁGINA DE CADASTRO DE CLIENTES</t>
   </si>
   <si>
-    <t xml:space="preserve">RF 03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">O SISTEMA DEVERÁ CONTER UMA
+    <t>RF 03</t>
+  </si>
+  <si>
+    <t>O SISTEMA DEVERÁ CONTER UMA
 PÁGINA DE CADASTRO DE PRODUTOS</t>
   </si>
   <si>
-    <t xml:space="preserve">RF 04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">O SISTEMA DEVERÁ CONTER UMA PÁGINA
+    <t>RF 04</t>
+  </si>
+  <si>
+    <t>O SISTEMA DEVERÁ CONTER UMA PÁGINA
 PARA PROCURAR E VISUALIZAR O ESTOQUE DE PRODUTOS</t>
   </si>
   <si>
-    <t xml:space="preserve">RF 05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">O SISTEMA DEVERÁ CONTER UMA
+    <t>RF 05</t>
+  </si>
+  <si>
+    <t>O SISTEMA DEVERÁ CONTER UMA
 PÁGINA HOME COM RESUMOS DAS INFORMAÇÕES DA EMPRESA, VENDAS, LUCROS E CUSTOS</t>
   </si>
   <si>
-    <t xml:space="preserve">RF 06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">O SISTEMA DEVERÁ CONTER UMA
+    <t>RF 06</t>
+  </si>
+  <si>
+    <t>O SISTEMA DEVERÁ CONTER UMA
 PÁGINA ONDE DÊ PARA VISUALIZAR,
 ATUALIZAR, LISTAR OU DELETAR OS DADOS DOS FUNCIONÁRIOS</t>
   </si>
   <si>
-    <t xml:space="preserve">RF 07</t>
-  </si>
-  <si>
-    <t xml:space="preserve">O SISTEMA DEVERÁ INTEGRAR-SE A API`s EXTERNAS PARA CONSULTA DE DADOS RELEVANTES AO NEGÓCIO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RF 08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">O SISTEMA DEVERÁ CONTER UM BOTÃO DE LOGOUT PARA O USUÁRIO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IMPORTANTE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RF 09</t>
-  </si>
-  <si>
-    <t xml:space="preserve">O SISTEMA DEVERÁ CONTER UMA PÁGINA DE INFORMAÇÕES GERAL, ONDE O USUÁRIO PODE VIZUALIZAR OS DADOS COM MAIS DETALHES</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RF 10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">O SISTEMA DEVERÁ PERMITIR EDITAÇÃO DE DADOS CADASTRADOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">REQUISITOS NÃO FUNCIONAIS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RNF 01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">O SISTEMA DEVE CONTER
+    <t>RF 07</t>
+  </si>
+  <si>
+    <t>O SISTEMA DEVERÁ INTEGRAR-SE A API`s EXTERNAS PARA CONSULTA DE DADOS RELEVANTES AO NEGÓCIO</t>
+  </si>
+  <si>
+    <t>RF 08</t>
+  </si>
+  <si>
+    <t>O SISTEMA DEVERÁ CONTER UM BOTÃO DE LOGOUT PARA O USUÁRIO</t>
+  </si>
+  <si>
+    <t>IMPORTANTE</t>
+  </si>
+  <si>
+    <t>RF 09</t>
+  </si>
+  <si>
+    <t>O SISTEMA DEVERÁ CONTER UMA PÁGINA DE INFORMAÇÕES GERAL, ONDE O USUÁRIO PODE VIZUALIZAR OS DADOS COM MAIS DETALHES</t>
+  </si>
+  <si>
+    <t>RF 10</t>
+  </si>
+  <si>
+    <t>REQUISITOS NÃO FUNCIONAIS</t>
+  </si>
+  <si>
+    <t>RNF 01</t>
+  </si>
+  <si>
+    <t>O SISTEMA DEVE CONTER
 UMA INTERFACE INTUITIVA E FÁCIL PARA O USUÁRIO NAVEGAR</t>
   </si>
   <si>
-    <t xml:space="preserve">RNF 02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">O SISTEMA DEVE ESTAR ONLINE A
+    <t>RNF 02</t>
+  </si>
+  <si>
+    <t>O SISTEMA DEVE ESTAR ONLINE A
 QUALQUER MOMENTO</t>
   </si>
   <si>
-    <t xml:space="preserve">RNF 03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">O SISTEMA DEVE CONTER COM UM
+    <t>RNF 03</t>
+  </si>
+  <si>
+    <t>O SISTEMA DEVE CONTER COM UM
 SUPORTE DISPONÍVEL POR 24 HORAS</t>
   </si>
   <si>
-    <t xml:space="preserve">DESEJÁVEL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RNF 04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">O SISTEMA DEVE TER UM CARREGAMENTO
+    <t>DESEJÁVEL</t>
+  </si>
+  <si>
+    <t>RNF 04</t>
+  </si>
+  <si>
+    <t>O SISTEMA DEVE TER UM CARREGAMENTO
 MENOR QUE 3 SEGUNDO</t>
   </si>
   <si>
-    <t xml:space="preserve">RNF 05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">O SISTEMA DEVE SER COMPATÍVEL
+    <t>RNF 05</t>
+  </si>
+  <si>
+    <t>O SISTEMA DEVE SER COMPATÍVEL
 COM DIFERENTES DISPOSITIVOS
 (DESKTOP, TABLET, MOBILE)</t>
   </si>
   <si>
-    <t xml:space="preserve">RNF 06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">O SISTEMA DEVE GARANTIR A
+    <t>RNF 06</t>
+  </si>
+  <si>
+    <t>O SISTEMA DEVE GARANTIR A
 SEGURANÇA DAS INFORMAÇÕES
 POR MEIO DE AUTENTICAÇÃO E
 CONTROLE DE ACESSO</t>
+  </si>
+  <si>
+    <t>O SISTEMA DEVERÁ PERMITIR EDITAÇÃO DE DADOS CADASTRADOS DE CADA PRODUTO</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="General"/>
-  </numFmts>
-  <fonts count="9">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <b val="true"/>
+      <b/>
       <sz val="12"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
+      <b/>
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
@@ -218,11 +201,10 @@
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
+      <b/>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -253,88 +235,57 @@
     </fill>
   </fills>
   <borders count="2">
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="20">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="8">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
-  <cellStyles count="6">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="15" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
-    <cellStyle name="Currency" xfId="17" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
-    <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -393,62 +344,78 @@
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF333399"/>
       <rgbColor rgb="FF333333"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
     </indexedColors>
   </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
     <a:clrScheme name="LibreOffice">
       <a:dk1>
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="18a303"/>
+        <a:srgbClr val="18A303"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="0369a3"/>
+        <a:srgbClr val="0369A3"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a33e03"/>
+        <a:srgbClr val="A33E03"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8e03a3"/>
+        <a:srgbClr val="8E03A3"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="c99c00"/>
+        <a:srgbClr val="C99C00"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="c9211e"/>
+        <a:srgbClr val="C9211E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ee"/>
+        <a:srgbClr val="0000EE"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="551a8b"/>
+        <a:srgbClr val="551A8B"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
-        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
-        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Arial"/>
+        <a:ea typeface="DejaVu Sans"/>
+        <a:cs typeface="DejaVu Sans"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
-        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
-        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Arial"/>
+        <a:ea typeface="DejaVu Sans"/>
+        <a:cs typeface="DejaVu Sans"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme>
@@ -501,37 +468,36 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B1:H22"/>
-  <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="12.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="8.34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="42.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="22.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="11.56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="11.22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="39.22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="18.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="8.77"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="11" style="0" width="11.56"/>
+    <col min="2" max="2" width="8.33203125" customWidth="1"/>
+    <col min="3" max="3" width="42.6640625" customWidth="1"/>
+    <col min="4" max="4" width="22.109375" customWidth="1"/>
+    <col min="5" max="5" width="11.5546875" customWidth="1"/>
+    <col min="6" max="6" width="11.21875" customWidth="1"/>
+    <col min="7" max="7" width="39.21875" customWidth="1"/>
+    <col min="8" max="8" width="18.88671875" customWidth="1"/>
+    <col min="10" max="10" width="8.77734375" customWidth="1"/>
+    <col min="11" max="16" width="11.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="true" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="2" s="1" customFormat="true" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B2" s="2" t="s">
+    <row r="1" spans="2:8" s="2" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="2:8" s="2" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-    </row>
-    <row r="3" s="1" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+    </row>
+    <row r="3" spans="2:8" s="2" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="3" t="s">
         <v>1</v>
       </c>
@@ -542,7 +508,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" s="1" customFormat="true" ht="52.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="4" spans="2:8" s="2" customFormat="1" ht="52.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="4" t="s">
         <v>4</v>
       </c>
@@ -553,7 +519,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" s="1" customFormat="true" ht="43" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" spans="2:8" s="2" customFormat="1" ht="43.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="4" t="s">
         <v>7</v>
       </c>
@@ -564,7 +530,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" s="1" customFormat="true" ht="62.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" spans="2:8" s="2" customFormat="1" ht="62.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="4" t="s">
         <v>9</v>
       </c>
@@ -576,7 +542,7 @@
       </c>
       <c r="G6" s="7"/>
     </row>
-    <row r="7" s="1" customFormat="true" ht="63" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="7" spans="2:8" s="2" customFormat="1" ht="63" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="4" t="s">
         <v>11</v>
       </c>
@@ -587,7 +553,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" s="1" customFormat="true" ht="69" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" spans="2:8" s="2" customFormat="1" ht="69" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="4" t="s">
         <v>13</v>
       </c>
@@ -598,7 +564,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" s="1" customFormat="true" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="9" spans="2:8" s="2" customFormat="1" ht="72" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="4" t="s">
         <v>15</v>
       </c>
@@ -609,7 +575,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="10" s="1" customFormat="true" ht="67.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" spans="2:8" s="2" customFormat="1" ht="67.650000000000006" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="4" t="s">
         <v>17</v>
       </c>
@@ -620,7 +586,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="11" s="1" customFormat="true" ht="55.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="11" spans="2:8" s="2" customFormat="1" ht="55.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="4" t="s">
         <v>19</v>
       </c>
@@ -631,7 +597,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" s="1" customFormat="true" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="12" spans="2:8" s="2" customFormat="1" ht="66" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="4" t="s">
         <v>22</v>
       </c>
@@ -642,25 +608,25 @@
         <v>6</v>
       </c>
     </row>
-    <row r="13" s="1" customFormat="true" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="13" spans="2:8" s="2" customFormat="1" ht="66" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="4" t="s">
         <v>24</v>
       </c>
       <c r="C13" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="14" spans="2:8" s="2" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F14" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="D13" s="6" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="14" s="1" customFormat="true" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="F14" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="G14" s="2"/>
-      <c r="H14" s="2"/>
-    </row>
-    <row r="15" s="1" customFormat="true" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="G14" s="1"/>
+      <c r="H14" s="1"/>
+    </row>
+    <row r="15" spans="2:8" s="2" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F15" s="3" t="s">
         <v>1</v>
       </c>
@@ -671,84 +637,79 @@
         <v>3</v>
       </c>
     </row>
-    <row r="16" s="1" customFormat="true" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="16" spans="2:8" s="2" customFormat="1" ht="54" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F16" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G16" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="G16" s="5" t="s">
+      <c r="H16" s="6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="17" spans="6:8" s="2" customFormat="1" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F17" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="H16" s="6" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="17" s="1" customFormat="true" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="F17" s="4" t="s">
+      <c r="G17" s="5" t="s">
         <v>29</v>
-      </c>
-      <c r="G17" s="5" t="s">
-        <v>30</v>
       </c>
       <c r="H17" s="6" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="18" s="1" customFormat="true" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" spans="6:8" s="2" customFormat="1" ht="60" x14ac:dyDescent="0.25">
       <c r="F18" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="G18" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="G18" s="5" t="s">
+      <c r="H18" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="H18" s="6" t="s">
+    </row>
+    <row r="19" spans="6:8" s="2" customFormat="1" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F19" s="4" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="19" s="1" customFormat="true" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="F19" s="4" t="s">
+      <c r="G19" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="G19" s="5" t="s">
+      <c r="H19" s="6" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="20" spans="6:8" s="2" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+      <c r="F20" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="H19" s="6" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="20" s="1" customFormat="true" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F20" s="4" t="s">
+      <c r="G20" s="5" t="s">
         <v>36</v>
-      </c>
-      <c r="G20" s="5" t="s">
-        <v>37</v>
       </c>
       <c r="H20" s="6" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="21" s="1" customFormat="true" ht="69" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="21" spans="6:8" s="2" customFormat="1" ht="69" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F21" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="G21" s="5" t="s">
         <v>38</v>
-      </c>
-      <c r="G21" s="5" t="s">
-        <v>39</v>
       </c>
       <c r="H21" s="6" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="22" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="22" spans="6:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="B2:D2"/>
     <mergeCell ref="F14:H14"/>
   </mergeCells>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.511805555555556" right="0.511805555555556" top="0.7875" bottom="0.7875" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageMargins left="0.51180555555555596" right="0.51180555555555596" top="0.78749999999999998" bottom="0.78749999999999998" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
</xml_diff>